<commit_message>
LIB07 update 2026-04-12 19:25:56 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,24 +463,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,24 +490,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -517,24 +517,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -544,24 +544,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -571,24 +571,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -598,24 +598,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -625,24 +625,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -652,24 +652,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -684,19 +684,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -711,19 +711,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -738,19 +738,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,90</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 a.m.</t>
+          <t>12/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,85</t>
+          <t>28,63</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -792,19 +792,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.000,17</t>
+          <t>999,63</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11/04/2026 11:00 p.m.</t>
+          <t>12/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,68</t>
+          <t>28,85</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -819,19 +819,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.000,62</t>
+          <t>1.000,17</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11/04/2026 10:00 p.m.</t>
+          <t>11/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,90</t>
+          <t>28,68</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -846,19 +846,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.000,86</t>
+          <t>1.000,62</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11/04/2026 09:00 p.m.</t>
+          <t>11/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>28,90</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -873,19 +873,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.000,51</t>
+          <t>1.000,86</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11/04/2026 08:00 p.m.</t>
+          <t>11/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>29,48</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,19 +900,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>999,90</t>
+          <t>1.000,51</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11/04/2026 07:00 p.m.</t>
+          <t>11/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>29,93</t>
+          <t>29,48</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,19 +927,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>999,44</t>
+          <t>999,90</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11/04/2026 06:00 p.m.</t>
+          <t>11/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>30,88</t>
+          <t>29,93</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -949,24 +949,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,13</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>998,82</t>
+          <t>999,44</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11/04/2026 05:00 p.m.</t>
+          <t>11/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>32,86</t>
+          <t>30,88</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -976,24 +976,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,46</t>
+          <t>0,13</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>998,01</t>
+          <t>998,82</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11/04/2026 04:00 p.m.</t>
+          <t>11/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>33,39</t>
+          <t>32,86</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1003,24 +1003,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,85</t>
+          <t>0,46</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>997,59</t>
+          <t>998,01</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11/04/2026 03:00 p.m.</t>
+          <t>11/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>33,79</t>
+          <t>33,39</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1030,24 +1030,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1,15</t>
+          <t>0,85</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>997,83</t>
+          <t>997,59</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/04/2026 02:00 p.m.</t>
+          <t>11/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>33,93</t>
+          <t>33,79</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1062,19 +1062,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>998,64</t>
+          <t>997,83</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/04/2026 01:00 p.m.</t>
+          <t>11/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>34,99</t>
+          <t>33,93</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1084,24 +1084,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1,35</t>
+          <t>1,15</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>999,23</t>
+          <t>998,64</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/04/2026 12:00 p.m.</t>
+          <t>11/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>35,38</t>
+          <t>34,99</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1111,12 +1111,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1,13</t>
+          <t>1,35</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.000,03</t>
+          <t>999,23</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 12:22:27 p.m.</t>
+          <t>12/04/2026 01:22:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>36,00</t>
+          <t>36,58</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>34,95</t>
+          <t>36,25</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>19,99</t>
+          <t>20,27</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>41,83</t>
+          <t>39,62</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>38,05</t>
+          <t>36,43</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>70,91</t>
+          <t>66,27</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>49,39</t>
+          <t>51,37</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>37,51</t>
+          <t>38,82</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 update 2026-04-12 20:00:34 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 01:22:27 p.m.</t>
+          <t>12/04/2026 01:52:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>36,25</t>
+          <t>35,50</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>20,27</t>
+          <t>19,46</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>39,62</t>
+          <t>39,26</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>36,43</t>
+          <t>40,93</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>66,27</t>
+          <t>53,12</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>51,37</t>
+          <t>54,18</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>38,82</t>
+          <t>37,70</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 update 2026-04-12 20:54:15 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,24 +463,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,24 +490,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -517,24 +517,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -544,24 +544,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -571,24 +571,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -598,24 +598,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -625,24 +625,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -652,24 +652,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -679,24 +679,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -711,19 +711,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -738,19 +738,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -792,19 +792,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,90</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 a.m.</t>
+          <t>12/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,85</t>
+          <t>28,63</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -819,19 +819,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.000,17</t>
+          <t>999,63</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11/04/2026 11:00 p.m.</t>
+          <t>12/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,68</t>
+          <t>28,85</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -846,19 +846,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.000,62</t>
+          <t>1.000,17</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11/04/2026 10:00 p.m.</t>
+          <t>11/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,90</t>
+          <t>28,68</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -873,19 +873,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.000,86</t>
+          <t>1.000,62</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11/04/2026 09:00 p.m.</t>
+          <t>11/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>28,90</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,19 +900,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.000,51</t>
+          <t>1.000,86</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11/04/2026 08:00 p.m.</t>
+          <t>11/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>29,48</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,19 +927,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>999,90</t>
+          <t>1.000,51</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11/04/2026 07:00 p.m.</t>
+          <t>11/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>29,93</t>
+          <t>29,48</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -954,19 +954,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>999,44</t>
+          <t>999,90</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11/04/2026 06:00 p.m.</t>
+          <t>11/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>30,88</t>
+          <t>29,93</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -976,24 +976,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,13</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>998,82</t>
+          <t>999,44</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11/04/2026 05:00 p.m.</t>
+          <t>11/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>32,86</t>
+          <t>30,88</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1003,24 +1003,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,46</t>
+          <t>0,13</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>998,01</t>
+          <t>998,82</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11/04/2026 04:00 p.m.</t>
+          <t>11/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>33,39</t>
+          <t>32,86</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1030,24 +1030,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,85</t>
+          <t>0,46</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>997,59</t>
+          <t>998,01</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/04/2026 03:00 p.m.</t>
+          <t>11/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>33,79</t>
+          <t>33,39</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1057,24 +1057,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1,15</t>
+          <t>0,85</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>997,83</t>
+          <t>997,59</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/04/2026 02:00 p.m.</t>
+          <t>11/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>33,93</t>
+          <t>33,79</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1089,19 +1089,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>998,64</t>
+          <t>997,83</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/04/2026 01:00 p.m.</t>
+          <t>11/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>34,99</t>
+          <t>33,93</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1111,12 +1111,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1,35</t>
+          <t>1,15</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>999,23</t>
+          <t>998,64</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 01:52:27 p.m.</t>
+          <t>12/04/2026 02:52:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>35,50</t>
+          <t>35,36</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>19,46</t>
+          <t>20,08</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>39,26</t>
+          <t>41,12</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>40,93</t>
+          <t>28,36</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>53,12</t>
+          <t>74,71</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>54,18</t>
+          <t>48,78</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>37,70</t>
+          <t>37,91</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 update 2026-04-12 21:40:31 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,24 +463,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,24 +490,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -517,24 +517,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -544,24 +544,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -571,24 +571,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -598,24 +598,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -625,24 +625,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -652,24 +652,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -679,24 +679,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -706,24 +706,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -738,19 +738,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -792,19 +792,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -819,19 +819,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,90</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 a.m.</t>
+          <t>12/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,85</t>
+          <t>28,63</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -846,19 +846,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.000,17</t>
+          <t>999,63</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11/04/2026 11:00 p.m.</t>
+          <t>12/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,68</t>
+          <t>28,85</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -873,19 +873,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.000,62</t>
+          <t>1.000,17</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11/04/2026 10:00 p.m.</t>
+          <t>11/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,90</t>
+          <t>28,68</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,19 +900,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.000,86</t>
+          <t>1.000,62</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11/04/2026 09:00 p.m.</t>
+          <t>11/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>28,90</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,19 +927,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.000,51</t>
+          <t>1.000,86</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11/04/2026 08:00 p.m.</t>
+          <t>11/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>29,48</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -954,19 +954,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>999,90</t>
+          <t>1.000,51</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11/04/2026 07:00 p.m.</t>
+          <t>11/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>29,93</t>
+          <t>29,48</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -981,19 +981,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>999,44</t>
+          <t>999,90</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11/04/2026 06:00 p.m.</t>
+          <t>11/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>30,88</t>
+          <t>29,93</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1003,24 +1003,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,13</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>998,82</t>
+          <t>999,44</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11/04/2026 05:00 p.m.</t>
+          <t>11/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>32,86</t>
+          <t>30,88</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1030,24 +1030,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,46</t>
+          <t>0,13</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>998,01</t>
+          <t>998,82</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/04/2026 04:00 p.m.</t>
+          <t>11/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>33,39</t>
+          <t>32,86</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1057,24 +1057,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,85</t>
+          <t>0,46</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>997,59</t>
+          <t>998,01</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/04/2026 03:00 p.m.</t>
+          <t>11/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>33,79</t>
+          <t>33,39</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1084,24 +1084,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1,15</t>
+          <t>0,85</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>997,83</t>
+          <t>997,59</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/04/2026 02:00 p.m.</t>
+          <t>11/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>33,93</t>
+          <t>33,79</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>998,64</t>
+          <t>997,83</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 02:52:27 p.m.</t>
+          <t>12/04/2026 03:32:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>35,36</t>
+          <t>34,49</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>20,08</t>
+          <t>19,26</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>41,12</t>
+          <t>41,00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>28,36</t>
+          <t>33,59</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>74,71</t>
+          <t>50,54</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>48,78</t>
+          <t>45,97</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>37,91</t>
+          <t>36,70</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 update 2026-04-12 22:04:36 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,24 +463,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,24 +490,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -517,24 +517,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -544,24 +544,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -571,24 +571,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -598,24 +598,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -625,24 +625,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -652,24 +652,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -679,24 +679,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -706,24 +706,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -733,24 +733,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -765,19 +765,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -792,19 +792,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -819,19 +819,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -846,19 +846,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,90</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 a.m.</t>
+          <t>12/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,85</t>
+          <t>28,63</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -873,19 +873,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.000,17</t>
+          <t>999,63</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11/04/2026 11:00 p.m.</t>
+          <t>12/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,68</t>
+          <t>28,85</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,19 +900,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.000,62</t>
+          <t>1.000,17</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11/04/2026 10:00 p.m.</t>
+          <t>11/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28,90</t>
+          <t>28,68</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,19 +927,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.000,86</t>
+          <t>1.000,62</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11/04/2026 09:00 p.m.</t>
+          <t>11/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>28,90</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -954,19 +954,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.000,51</t>
+          <t>1.000,86</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11/04/2026 08:00 p.m.</t>
+          <t>11/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>29,48</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -981,19 +981,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>999,90</t>
+          <t>1.000,51</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11/04/2026 07:00 p.m.</t>
+          <t>11/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>29,93</t>
+          <t>29,48</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1008,19 +1008,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>999,44</t>
+          <t>999,90</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11/04/2026 06:00 p.m.</t>
+          <t>11/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>30,88</t>
+          <t>29,93</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1030,24 +1030,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,13</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>998,82</t>
+          <t>999,44</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/04/2026 05:00 p.m.</t>
+          <t>11/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>32,86</t>
+          <t>30,88</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1057,24 +1057,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,46</t>
+          <t>0,13</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>998,01</t>
+          <t>998,82</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/04/2026 04:00 p.m.</t>
+          <t>11/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>33,39</t>
+          <t>32,86</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1084,24 +1084,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,85</t>
+          <t>0,46</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>997,59</t>
+          <t>998,01</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/04/2026 03:00 p.m.</t>
+          <t>11/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>33,79</t>
+          <t>33,39</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1111,12 +1111,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1,15</t>
+          <t>0,85</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>997,83</t>
+          <t>997,59</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 03:32:27 p.m.</t>
+          <t>12/04/2026 04:02:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>34,49</t>
+          <t>34,78</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>19,26</t>
+          <t>19,56</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>41,00</t>
+          <t>41,10</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>33,59</t>
+          <t>27,00</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>50,54</t>
+          <t>71,85</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>45,97</t>
+          <t>39,78</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>36,70</t>
+          <t>37,14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 update 2026-04-12 22:56:59 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 04:22:27 p.m.</t>
+          <t>12/04/2026 04:52:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>33,64</t>
+          <t>33,03</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>20,08</t>
+          <t>19,49</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>45,24</t>
+          <t>45,13</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>31,79</t>
+          <t>27,63</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>50,57</t>
+          <t>61,36</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>38,20</t>
+          <t>34,99</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>36,39</t>
+          <t>35,52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-12 23:17:53 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,24 +463,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,24 +490,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -517,24 +517,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -544,24 +544,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -571,24 +571,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -598,24 +598,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -625,24 +625,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -652,24 +652,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -679,24 +679,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -706,24 +706,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -733,24 +733,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -760,24 +760,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -792,19 +792,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -819,19 +819,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -846,19 +846,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -873,19 +873,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,90</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 a.m.</t>
+          <t>12/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,85</t>
+          <t>28,63</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,19 +900,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.000,17</t>
+          <t>999,63</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11/04/2026 11:00 p.m.</t>
+          <t>12/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28,68</t>
+          <t>28,85</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,19 +927,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.000,62</t>
+          <t>1.000,17</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11/04/2026 10:00 p.m.</t>
+          <t>11/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>28,90</t>
+          <t>28,68</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -954,19 +954,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.000,86</t>
+          <t>1.000,62</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11/04/2026 09:00 p.m.</t>
+          <t>11/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>28,90</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -981,19 +981,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.000,51</t>
+          <t>1.000,86</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11/04/2026 08:00 p.m.</t>
+          <t>11/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>29,48</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1008,19 +1008,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>999,90</t>
+          <t>1.000,51</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11/04/2026 07:00 p.m.</t>
+          <t>11/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>29,93</t>
+          <t>29,48</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1035,19 +1035,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>999,44</t>
+          <t>999,90</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/04/2026 06:00 p.m.</t>
+          <t>11/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>30,88</t>
+          <t>29,93</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1057,24 +1057,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,13</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>998,82</t>
+          <t>999,44</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/04/2026 05:00 p.m.</t>
+          <t>11/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>32,86</t>
+          <t>30,88</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1084,24 +1084,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,46</t>
+          <t>0,13</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>998,01</t>
+          <t>998,82</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/04/2026 04:00 p.m.</t>
+          <t>11/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>33,39</t>
+          <t>32,86</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1111,12 +1111,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,85</t>
+          <t>0,46</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>997,59</t>
+          <t>998,01</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 04:52:27 p.m.</t>
+          <t>12/04/2026 05:12:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>33,03</t>
+          <t>32,70</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>19,49</t>
+          <t>19,42</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>45,13</t>
+          <t>45,76</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>27,63</t>
+          <t>24,99</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>61,36</t>
+          <t>80,00</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>34,99</t>
+          <t>33,19</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>35,52</t>
+          <t>35,20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-12 23:52:05 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 05:12:27 p.m.</t>
+          <t>12/04/2026 05:42:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>32,70</t>
+          <t>31,50</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>19,42</t>
+          <t>19,66</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>45,76</t>
+          <t>49,73</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>28,87</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>80,00</t>
+          <t>67,59</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>33,19</t>
+          <t>39,17</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>35,20</t>
+          <t>29,47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 00:12:02 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,24 +463,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,24 +490,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -517,24 +517,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -544,24 +544,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -571,24 +571,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -598,24 +598,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -625,24 +625,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -652,24 +652,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -679,24 +679,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -706,24 +706,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -733,24 +733,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -760,24 +760,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -787,24 +787,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -819,19 +819,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -846,19 +846,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -873,19 +873,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,19 +900,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,90</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 a.m.</t>
+          <t>12/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28,85</t>
+          <t>28,63</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,19 +927,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.000,17</t>
+          <t>999,63</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11/04/2026 11:00 p.m.</t>
+          <t>12/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>28,68</t>
+          <t>28,85</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -954,19 +954,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.000,62</t>
+          <t>1.000,17</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11/04/2026 10:00 p.m.</t>
+          <t>11/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>28,90</t>
+          <t>28,68</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -981,19 +981,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.000,86</t>
+          <t>1.000,62</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11/04/2026 09:00 p.m.</t>
+          <t>11/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>28,90</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1008,19 +1008,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.000,51</t>
+          <t>1.000,86</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11/04/2026 08:00 p.m.</t>
+          <t>11/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>29,48</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1035,19 +1035,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>999,90</t>
+          <t>1.000,51</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/04/2026 07:00 p.m.</t>
+          <t>11/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>29,93</t>
+          <t>29,48</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1062,19 +1062,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>999,44</t>
+          <t>999,90</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/04/2026 06:00 p.m.</t>
+          <t>11/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>30,88</t>
+          <t>29,93</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1084,24 +1084,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,13</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>998,82</t>
+          <t>999,44</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/04/2026 05:00 p.m.</t>
+          <t>11/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>32,86</t>
+          <t>30,88</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1111,12 +1111,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,46</t>
+          <t>0,13</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>998,01</t>
+          <t>998,82</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 05:42:27 p.m.</t>
+          <t>12/04/2026 06:02:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>31,50</t>
+          <t>30,97</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>19,66</t>
+          <t>19,76</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>49,73</t>
+          <t>51,55</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>28,87</t>
+          <t>28,52</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>67,59</t>
+          <t>73,64</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>39,17</t>
+          <t>38,59</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>29,47</t>
+          <t>29,12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 01:24:05 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,24 +463,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,24 +490,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -517,24 +517,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -544,24 +544,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -571,24 +571,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -598,24 +598,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -625,24 +625,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -652,24 +652,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -679,24 +679,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -706,24 +706,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -733,24 +733,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -760,24 +760,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -787,24 +787,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -814,24 +814,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -846,19 +846,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -873,19 +873,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,19 +900,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,19 +927,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,90</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 a.m.</t>
+          <t>12/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>28,85</t>
+          <t>28,63</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -954,19 +954,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.000,17</t>
+          <t>999,63</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11/04/2026 11:00 p.m.</t>
+          <t>12/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>28,68</t>
+          <t>28,85</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -981,19 +981,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.000,62</t>
+          <t>1.000,17</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11/04/2026 10:00 p.m.</t>
+          <t>11/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>28,90</t>
+          <t>28,68</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1008,19 +1008,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.000,86</t>
+          <t>1.000,62</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11/04/2026 09:00 p.m.</t>
+          <t>11/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>28,90</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1035,19 +1035,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.000,51</t>
+          <t>1.000,86</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/04/2026 08:00 p.m.</t>
+          <t>11/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>29,48</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1062,19 +1062,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>999,90</t>
+          <t>1.000,51</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/04/2026 07:00 p.m.</t>
+          <t>11/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>29,93</t>
+          <t>29,48</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1089,19 +1089,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>999,44</t>
+          <t>999,90</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/04/2026 06:00 p.m.</t>
+          <t>11/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>30,88</t>
+          <t>29,93</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1111,12 +1111,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,13</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>998,82</t>
+          <t>999,44</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 06:02:27 p.m.</t>
+          <t>12/04/2026 07:22:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>30,97</t>
+          <t>29,83</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>19,76</t>
+          <t>19,74</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>51,55</t>
+          <t>54,94</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>28,52</t>
+          <t>38,02</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>73,64</t>
+          <t>75,76</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>38,59</t>
+          <t>49,39</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>29,12</t>
+          <t>26,07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 01:53:27 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -1169,7 +1169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 07:22:27 p.m.</t>
+          <t>12/04/2026 07:52:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1262,37 +1262,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>29,83</t>
+          <t>29,62</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>19,74</t>
+          <t>19,17</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>54,94</t>
+          <t>53,71</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>38,02</t>
+          <t>29,30</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>75,76</t>
+          <t>78,12</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>49,39</t>
+          <t>40,00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>26,07</t>
+          <t>27,23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 03:04:42 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horarios" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuales_resumen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuales_inst" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,27 +430,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>temp</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>lluvia</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>radmax</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>presmb</t>
         </is>
@@ -448,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -468,19 +479,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -517,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -544,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -571,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -598,24 +609,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -625,24 +636,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -652,24 +663,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -679,24 +690,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -706,24 +717,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -733,24 +744,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -760,24 +771,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -787,24 +798,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -814,24 +825,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -841,24 +852,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -868,24 +879,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -900,19 +911,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -927,19 +938,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -954,19 +965,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 a.m.</t>
+          <t>12/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>28,85</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -981,19 +992,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.000,17</t>
+          <t>998,90</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11/04/2026 11:00 p.m.</t>
+          <t>12/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>28,68</t>
+          <t>28,63</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1008,19 +1019,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.000,62</t>
+          <t>999,63</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>28,90</t>
+          <t>28,85</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1035,19 +1046,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.000,86</t>
+          <t>1.000,17</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/04/2026 09:00 p.m.</t>
+          <t>11/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>28,68</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1062,19 +1073,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.000,51</t>
+          <t>1.000,62</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/04/2026 08:00 p.m.</t>
+          <t>11/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>29,48</t>
+          <t>28,90</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1089,19 +1100,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>999,90</t>
+          <t>1.000,86</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/04/2026 07:00 p.m.</t>
+          <t>11/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>29,93</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1116,7 +1127,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>999,44</t>
+          <t>1.000,51</t>
         </is>
       </c>
     </row>
@@ -1135,32 +1146,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>vmax</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sumlluv</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>lluvayer</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>tmax</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>tmin</t>
         </is>
@@ -1169,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 07:52:27 p.m.</t>
+          <t>12/04/2026 09:02:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1195,104 +1206,6 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>26,51</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>fecha</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>temp</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>td</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>hr</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>velocidad</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>direccion</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>vpmax</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>stavg</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>12/04/2026</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>29,62</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>19,17</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>53,71</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>29,30</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>78,12</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>40,00</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>27,23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 04:55:53 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -479,19 +479,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -506,19 +506,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -533,19 +533,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -609,24 +609,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -636,24 +636,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -690,24 +690,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -717,24 +717,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -744,24 +744,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -771,24 +771,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -798,24 +798,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -825,24 +825,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -852,24 +852,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -879,24 +879,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -906,24 +906,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -938,19 +938,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -965,19 +965,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -992,19 +992,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1019,19 +1019,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,90</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 a.m.</t>
+          <t>12/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>28,85</t>
+          <t>28,63</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1046,19 +1046,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.000,17</t>
+          <t>999,63</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/04/2026 11:00 p.m.</t>
+          <t>12/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>28,68</t>
+          <t>28,85</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.000,62</t>
+          <t>1.000,17</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/04/2026 10:00 p.m.</t>
+          <t>11/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>28,90</t>
+          <t>28,68</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1100,19 +1100,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.000,86</t>
+          <t>1.000,62</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/04/2026 09:00 p.m.</t>
+          <t>11/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>28,90</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.000,51</t>
+          <t>1.000,86</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 09:02:27 p.m.</t>
+          <t>12/04/2026 10:52:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 07:14:24 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -479,19 +479,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -506,19 +506,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -533,19 +533,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -560,19 +560,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -609,24 +609,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -636,24 +636,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -690,24 +690,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -717,24 +717,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -744,24 +744,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -771,24 +771,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -798,24 +798,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -825,24 +825,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -852,24 +852,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -879,24 +879,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -906,24 +906,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -933,24 +933,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -960,24 +960,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -987,24 +987,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1019,19 +1019,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1046,19 +1046,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>28,85</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.000,17</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/04/2026 11:00 p.m.</t>
+          <t>12/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>28,68</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1100,19 +1100,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.000,62</t>
+          <t>998,90</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>28,90</t>
+          <t>28,63</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.000,86</t>
+          <t>999,63</t>
         </is>
       </c>
     </row>
@@ -1180,12 +1180,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12/04/2026 10:52:27 p.m.</t>
+          <t>13/04/2026 01:12:27 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>66,00</t>
+          <t>43,40</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1200,12 +1200,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>36,58</t>
+          <t>29,42</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>26,51</t>
+          <t>28,37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 09:14:24 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -479,19 +479,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -506,19 +506,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -533,19 +533,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -560,19 +560,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -587,19 +587,19 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -614,19 +614,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -641,19 +641,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -690,24 +690,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -717,24 +717,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -744,24 +744,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -771,24 +771,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -798,24 +798,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -825,24 +825,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -852,24 +852,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -879,24 +879,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -906,24 +906,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -933,24 +933,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -960,24 +960,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -987,24 +987,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1014,24 +1014,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1100,19 +1100,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>998,90</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 a.m.</t>
+          <t>12/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>28,63</t>
+          <t>28,47</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>999,63</t>
+          <t>998,38</t>
         </is>
       </c>
     </row>
@@ -1180,12 +1180,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 01:12:27 a.m.</t>
+          <t>13/04/2026 03:12:27 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>43,40</t>
+          <t>48,80</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>28,37</t>
+          <t>26,87</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 10:57:57 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -479,19 +479,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -506,19 +506,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -533,19 +533,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -560,19 +560,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -587,19 +587,19 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -614,19 +614,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -641,19 +641,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -668,19 +668,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -695,19 +695,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -717,24 +717,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -744,24 +744,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -771,24 +771,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -798,24 +798,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -825,24 +825,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -852,24 +852,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -879,24 +879,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -906,24 +906,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -933,24 +933,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -960,24 +960,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -987,24 +987,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1014,24 +1014,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>27,22</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1100,19 +1100,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>998,93</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 a.m.</t>
+          <t>12/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>28,47</t>
+          <t>28,01</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>998,38</t>
+          <t>998,25</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 03:12:27 a.m.</t>
+          <t>13/04/2026 04:52:27 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 12:07:31 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -506,19 +506,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -533,19 +533,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -560,19 +560,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -587,19 +587,19 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -614,19 +614,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -641,19 +641,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -668,19 +668,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -695,19 +695,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -722,19 +722,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -744,24 +744,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -771,24 +771,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -798,24 +798,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -825,24 +825,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -852,24 +852,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -879,24 +879,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -906,24 +906,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -933,24 +933,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -960,24 +960,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -987,24 +987,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1014,24 +1014,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 a.m.</t>
+          <t>12/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>27,22</t>
+          <t>29,11</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>998,93</t>
+          <t>999,70</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 a.m.</t>
+          <t>12/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>28,01</t>
+          <t>28,31</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,04</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>998,25</t>
+          <t>999,22</t>
         </is>
       </c>
     </row>
@@ -1180,12 +1180,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 04:52:27 a.m.</t>
+          <t>13/04/2026 06:02:27 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>48,80</t>
+          <t>51,40</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 14:06:18 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 06:00 a.m.</t>
+          <t>13/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>28,51</t>
+          <t>30,87</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>999,89</t>
+          <t>1.001,49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 a.m.</t>
+          <t>13/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>28,49</t>
+          <t>29,25</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>999,42</t>
+          <t>1.000,76</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -528,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -560,19 +560,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -587,19 +587,19 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -614,19 +614,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -641,19 +641,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -668,19 +668,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -695,19 +695,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -722,19 +722,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -749,19 +749,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -776,19 +776,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -798,24 +798,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -825,24 +825,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -852,24 +852,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -879,24 +879,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -906,24 +906,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -933,24 +933,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -960,24 +960,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -987,24 +987,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1014,24 +1014,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>29,11</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>999,70</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 a.m.</t>
+          <t>12/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>28,31</t>
+          <t>30,46</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,44</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>999,22</t>
+          <t>1.000,69</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 06:02:27 a.m.</t>
+          <t>13/04/2026 08:02:27 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>29,42</t>
+          <t>31,82</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 15:43:44 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 08:00 a.m.</t>
+          <t>13/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>30,87</t>
+          <t>31,69</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>0,78</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.001,49</t>
+          <t>1.001,82</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 07:00 a.m.</t>
+          <t>13/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>29,25</t>
+          <t>30,87</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.000,76</t>
+          <t>1.001,49</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 06:00 a.m.</t>
+          <t>13/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>28,51</t>
+          <t>29,25</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -528,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>999,89</t>
+          <t>1.000,76</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>28,49</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>999,42</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -587,19 +587,19 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -614,19 +614,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -641,19 +641,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -668,19 +668,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -695,19 +695,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -722,19 +722,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -749,19 +749,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -776,19 +776,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -803,19 +803,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -830,19 +830,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -852,24 +852,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -879,24 +879,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -906,24 +906,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -933,24 +933,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -960,24 +960,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -987,24 +987,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1014,24 +1014,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 a.m.</t>
+          <t>12/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>30,46</t>
+          <t>31,28</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,44</t>
+          <t>0,64</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.000,69</t>
+          <t>1.001,12</t>
         </is>
       </c>
     </row>
@@ -1180,12 +1180,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 08:02:27 a.m.</t>
+          <t>13/04/2026 09:42:27 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>51,40</t>
+          <t>65,60</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>31,82</t>
+          <t>33,32</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 16:47:36 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 09:00 a.m.</t>
+          <t>13/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>31,69</t>
+          <t>32,79</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,78</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.001,82</t>
+          <t>1.001,88</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 08:00 a.m.</t>
+          <t>13/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30,87</t>
+          <t>31,69</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>0,78</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.001,49</t>
+          <t>1.001,82</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 07:00 a.m.</t>
+          <t>13/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>29,25</t>
+          <t>30,87</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -528,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.000,76</t>
+          <t>1.001,49</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 06:00 a.m.</t>
+          <t>13/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>28,51</t>
+          <t>29,25</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>999,89</t>
+          <t>1.000,76</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>28,49</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>999,42</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -614,19 +614,19 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -641,19 +641,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -668,19 +668,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -695,19 +695,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -722,19 +722,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -749,19 +749,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -776,19 +776,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -803,19 +803,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -830,19 +830,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -857,19 +857,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -879,24 +879,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -906,24 +906,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -933,24 +933,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -960,24 +960,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -987,24 +987,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1014,24 +1014,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 a.m.</t>
+          <t>12/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>31,28</t>
+          <t>32,84</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,64</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.001,12</t>
+          <t>1.000,91</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 09:42:27 a.m.</t>
+          <t>13/04/2026 10:22:27 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>33,32</t>
+          <t>34,09</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 17:47:09 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 10:00 a.m.</t>
+          <t>13/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>32,79</t>
+          <t>33,85</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>1,05</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.001,88</t>
+          <t>1.001,52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 09:00 a.m.</t>
+          <t>13/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>31,69</t>
+          <t>32,79</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,78</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.001,82</t>
+          <t>1.001,88</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 08:00 a.m.</t>
+          <t>13/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>30,87</t>
+          <t>31,69</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -528,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>0,78</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.001,49</t>
+          <t>1.001,82</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 07:00 a.m.</t>
+          <t>13/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29,25</t>
+          <t>30,87</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.000,76</t>
+          <t>1.001,49</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 06:00 a.m.</t>
+          <t>13/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>28,51</t>
+          <t>29,25</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>999,89</t>
+          <t>1.000,76</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>28,49</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -609,24 +609,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>999,42</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -641,19 +641,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -668,19 +668,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -695,19 +695,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -722,19 +722,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -749,19 +749,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -776,19 +776,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -803,19 +803,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -830,19 +830,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -857,19 +857,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -884,19 +884,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -906,24 +906,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -933,24 +933,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -960,24 +960,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -987,24 +987,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1014,24 +1014,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 a.m.</t>
+          <t>12/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>32,84</t>
+          <t>34,16</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,11</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.000,91</t>
+          <t>1.000,65</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 10:22:27 a.m.</t>
+          <t>13/04/2026 11:42:27 a.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>34,09</t>
+          <t>35,49</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 18:54:49 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 11:00 a.m.</t>
+          <t>13/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>33,85</t>
+          <t>34,70</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1,05</t>
+          <t>1,12</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.001,52</t>
+          <t>1.000,98</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 10:00 a.m.</t>
+          <t>13/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>32,79</t>
+          <t>33,85</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>1,05</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.001,88</t>
+          <t>1.001,52</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 09:00 a.m.</t>
+          <t>13/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>31,69</t>
+          <t>32,79</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -528,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,78</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.001,82</t>
+          <t>1.001,88</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 08:00 a.m.</t>
+          <t>13/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30,87</t>
+          <t>31,69</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>0,78</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.001,49</t>
+          <t>1.001,82</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 07:00 a.m.</t>
+          <t>13/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>29,25</t>
+          <t>30,87</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.000,76</t>
+          <t>1.001,49</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13/04/2026 06:00 a.m.</t>
+          <t>13/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>28,51</t>
+          <t>29,25</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -609,24 +609,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>999,89</t>
+          <t>1.000,76</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>28,49</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -636,24 +636,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>999,42</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -668,19 +668,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -695,19 +695,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -722,19 +722,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -749,19 +749,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -776,19 +776,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -803,19 +803,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -830,19 +830,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -857,19 +857,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -884,19 +884,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -911,19 +911,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -933,24 +933,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -960,24 +960,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -987,24 +987,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1014,24 +1014,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 a.m.</t>
+          <t>12/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>34,16</t>
+          <t>34,82</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1,11</t>
+          <t>1,14</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.000,65</t>
+          <t>1.000,28</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 11:42:27 a.m.</t>
+          <t>13/04/2026 12:22:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>35,49</t>
+          <t>35,62</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 mitigated update 2026-04-13 20:05:01 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 p.m.</t>
+          <t>13/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>34,70</t>
+          <t>35,00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1,12</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.000,98</t>
+          <t>1.000,05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 11:00 a.m.</t>
+          <t>13/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>33,85</t>
+          <t>34,70</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1,05</t>
+          <t>1,12</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.001,52</t>
+          <t>1.000,98</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 10:00 a.m.</t>
+          <t>13/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>32,79</t>
+          <t>33,85</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -528,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>1,05</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.001,88</t>
+          <t>1.001,52</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 09:00 a.m.</t>
+          <t>13/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>31,69</t>
+          <t>32,79</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,78</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.001,82</t>
+          <t>1.001,88</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 08:00 a.m.</t>
+          <t>13/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>30,87</t>
+          <t>31,69</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>0,78</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.001,49</t>
+          <t>1.001,82</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13/04/2026 07:00 a.m.</t>
+          <t>13/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>29,25</t>
+          <t>30,87</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -609,24 +609,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.000,76</t>
+          <t>1.001,49</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13/04/2026 06:00 a.m.</t>
+          <t>13/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>28,51</t>
+          <t>29,25</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -636,24 +636,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>999,89</t>
+          <t>1.000,76</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>28,49</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>999,42</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -695,19 +695,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -722,19 +722,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -749,19 +749,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -776,19 +776,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -803,19 +803,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -830,19 +830,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -857,19 +857,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -884,19 +884,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -911,19 +911,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -938,19 +938,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -960,24 +960,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -987,24 +987,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1014,24 +1014,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 01:00 p.m.</t>
+          <t>12/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>35,42</t>
+          <t>35,67</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1,19</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>999,77</t>
+          <t>998,95</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 12:00 p.m.</t>
+          <t>12/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>34,82</t>
+          <t>35,42</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1,14</t>
+          <t>1,19</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.000,28</t>
+          <t>999,77</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 12:22:27 p.m.</t>
+          <t>13/04/2026 01:22:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>35,62</t>
+          <t>36,16</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 update 2026-04-13 22:01:12 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 p.m.</t>
+          <t>13/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>35,41</t>
+          <t>35,31</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1,03</t>
+          <t>0,94</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>999,23</t>
+          <t>998,51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 p.m.</t>
+          <t>13/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>35,00</t>
+          <t>35,41</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,03</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.000,05</t>
+          <t>999,23</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 p.m.</t>
+          <t>13/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>34,70</t>
+          <t>35,00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -528,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1,12</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.000,98</t>
+          <t>1.000,05</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 11:00 a.m.</t>
+          <t>13/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>33,85</t>
+          <t>34,70</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1,05</t>
+          <t>1,12</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.001,52</t>
+          <t>1.000,98</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 10:00 a.m.</t>
+          <t>13/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>32,79</t>
+          <t>33,85</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>1,05</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.001,88</t>
+          <t>1.001,52</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13/04/2026 09:00 a.m.</t>
+          <t>13/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>31,69</t>
+          <t>32,79</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -609,24 +609,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,78</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.001,82</t>
+          <t>1.001,88</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13/04/2026 08:00 a.m.</t>
+          <t>13/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>30,87</t>
+          <t>31,69</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -636,24 +636,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>0,78</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.001,49</t>
+          <t>1.001,82</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13/04/2026 07:00 a.m.</t>
+          <t>13/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>29,25</t>
+          <t>30,87</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.000,76</t>
+          <t>1.001,49</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/04/2026 06:00 a.m.</t>
+          <t>13/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>28,51</t>
+          <t>29,25</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -690,24 +690,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>999,89</t>
+          <t>1.000,76</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28,49</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -717,24 +717,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>999,42</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -749,19 +749,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -776,19 +776,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -803,19 +803,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -830,19 +830,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -857,19 +857,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -884,19 +884,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -911,19 +911,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -938,19 +938,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -965,19 +965,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -992,19 +992,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1014,24 +1014,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 02:00 p.m.</t>
+          <t>12/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>35,67</t>
+          <t>35,33</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>998,95</t>
+          <t>998,44</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 02:22:27 p.m.</t>
+          <t>13/04/2026 03:22:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 update 2026-04-13 22:57:33 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 p.m.</t>
+          <t>13/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>35,31</t>
+          <t>34,51</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,94</t>
+          <t>0,62</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>998,51</t>
+          <t>998,21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 p.m.</t>
+          <t>13/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>35,41</t>
+          <t>35,31</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1,03</t>
+          <t>0,94</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>999,23</t>
+          <t>998,51</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 p.m.</t>
+          <t>13/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>35,00</t>
+          <t>35,41</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -528,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,03</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.000,05</t>
+          <t>999,23</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 p.m.</t>
+          <t>13/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>34,70</t>
+          <t>35,00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1,12</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.000,98</t>
+          <t>1.000,05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 11:00 a.m.</t>
+          <t>13/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>33,85</t>
+          <t>34,70</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1,05</t>
+          <t>1,12</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.001,52</t>
+          <t>1.000,98</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13/04/2026 10:00 a.m.</t>
+          <t>13/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>32,79</t>
+          <t>33,85</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -609,24 +609,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>1,05</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.001,88</t>
+          <t>1.001,52</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13/04/2026 09:00 a.m.</t>
+          <t>13/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>31,69</t>
+          <t>32,79</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -636,24 +636,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,78</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.001,82</t>
+          <t>1.001,88</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13/04/2026 08:00 a.m.</t>
+          <t>13/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>30,87</t>
+          <t>31,69</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>0,78</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.001,49</t>
+          <t>1.001,82</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/04/2026 07:00 a.m.</t>
+          <t>13/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>29,25</t>
+          <t>30,87</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -690,24 +690,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.000,76</t>
+          <t>1.001,49</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>13/04/2026 06:00 a.m.</t>
+          <t>13/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>28,51</t>
+          <t>29,25</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -717,24 +717,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>999,89</t>
+          <t>1.000,76</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,49</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -744,24 +744,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>999,42</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -776,19 +776,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -803,19 +803,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -830,19 +830,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -857,19 +857,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -884,19 +884,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -911,19 +911,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -938,19 +938,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -965,19 +965,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -992,19 +992,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1019,19 +1019,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1041,24 +1041,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 03:00 p.m.</t>
+          <t>12/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>35,33</t>
+          <t>34,84</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>0,67</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>998,44</t>
+          <t>998,32</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 03:22:27 p.m.</t>
+          <t>13/04/2026 04:52:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 update 2026-04-13 23:10:42 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 p.m.</t>
+          <t>13/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>34,51</t>
+          <t>33,36</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,62</t>
+          <t>0,40</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>998,21</t>
+          <t>998,16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 p.m.</t>
+          <t>13/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>35,31</t>
+          <t>34,51</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,94</t>
+          <t>0,62</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>998,51</t>
+          <t>998,21</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 p.m.</t>
+          <t>13/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>35,41</t>
+          <t>35,31</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -528,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1,03</t>
+          <t>0,94</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>999,23</t>
+          <t>998,51</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 p.m.</t>
+          <t>13/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>35,00</t>
+          <t>35,41</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>1,03</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.000,05</t>
+          <t>999,23</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 p.m.</t>
+          <t>13/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>34,70</t>
+          <t>35,00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1,12</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.000,98</t>
+          <t>1.000,05</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13/04/2026 11:00 a.m.</t>
+          <t>13/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>33,85</t>
+          <t>34,70</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -609,24 +609,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1,05</t>
+          <t>1,12</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.001,52</t>
+          <t>1.000,98</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13/04/2026 10:00 a.m.</t>
+          <t>13/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>32,79</t>
+          <t>33,85</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -636,24 +636,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>1,05</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.001,88</t>
+          <t>1.001,52</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13/04/2026 09:00 a.m.</t>
+          <t>13/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>31,69</t>
+          <t>32,79</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,78</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.001,82</t>
+          <t>1.001,88</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/04/2026 08:00 a.m.</t>
+          <t>13/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>30,87</t>
+          <t>31,69</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -690,24 +690,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>0,78</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.001,49</t>
+          <t>1.001,82</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>13/04/2026 07:00 a.m.</t>
+          <t>13/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>29,25</t>
+          <t>30,87</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -717,24 +717,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.000,76</t>
+          <t>1.001,49</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>13/04/2026 06:00 a.m.</t>
+          <t>13/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>28,51</t>
+          <t>29,25</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -744,24 +744,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>999,89</t>
+          <t>1.000,76</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,49</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -771,24 +771,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>999,42</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -803,19 +803,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -830,19 +830,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -857,19 +857,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -884,19 +884,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -911,19 +911,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -938,19 +938,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -965,19 +965,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -992,19 +992,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1019,19 +1019,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1046,19 +1046,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1068,24 +1068,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>31,93</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>999,54</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 04:00 p.m.</t>
+          <t>12/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>34,84</t>
+          <t>33,52</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,67</t>
+          <t>0,41</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>998,32</t>
+          <t>998,68</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 04:52:27 p.m.</t>
+          <t>13/04/2026 05:02:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
LIB07 update 2026-04-14 01:58:09 UTC
</commit_message>
<xml_diff>
--- a/salida_csv/lib07_tablas.xlsx
+++ b/salida_csv/lib07_tablas.xlsx
@@ -459,12 +459,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 p.m.</t>
+          <t>13/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>33,36</t>
+          <t>30,58</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -474,24 +474,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,40</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>998,16</t>
+          <t>999,36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 p.m.</t>
+          <t>13/04/2026 06:00 p.m.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>34,51</t>
+          <t>31,92</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -501,24 +501,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,62</t>
+          <t>0,16</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>998,21</t>
+          <t>998,60</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 p.m.</t>
+          <t>13/04/2026 05:00 p.m.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>35,31</t>
+          <t>33,36</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -528,24 +528,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,94</t>
+          <t>0,40</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>998,51</t>
+          <t>998,16</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 p.m.</t>
+          <t>13/04/2026 04:00 p.m.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>35,41</t>
+          <t>34,51</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -555,24 +555,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1,03</t>
+          <t>0,62</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>999,23</t>
+          <t>998,21</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 p.m.</t>
+          <t>13/04/2026 03:00 p.m.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>35,00</t>
+          <t>35,31</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,24 +582,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1,00</t>
+          <t>0,94</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.000,05</t>
+          <t>998,51</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 p.m.</t>
+          <t>13/04/2026 02:00 p.m.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>34,70</t>
+          <t>35,41</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -609,24 +609,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1,12</t>
+          <t>1,03</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.000,98</t>
+          <t>999,23</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13/04/2026 11:00 a.m.</t>
+          <t>13/04/2026 01:00 p.m.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>33,85</t>
+          <t>35,00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -636,24 +636,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1,05</t>
+          <t>1,00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.001,52</t>
+          <t>1.000,05</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13/04/2026 10:00 a.m.</t>
+          <t>13/04/2026 12:00 p.m.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>32,79</t>
+          <t>34,70</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -663,24 +663,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,95</t>
+          <t>1,12</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.001,88</t>
+          <t>1.000,98</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/04/2026 09:00 a.m.</t>
+          <t>13/04/2026 11:00 a.m.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>31,69</t>
+          <t>33,85</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -690,24 +690,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,78</t>
+          <t>1,05</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.001,82</t>
+          <t>1.001,52</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>13/04/2026 08:00 a.m.</t>
+          <t>13/04/2026 10:00 a.m.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>30,87</t>
+          <t>32,79</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -717,24 +717,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,43</t>
+          <t>0,95</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.001,49</t>
+          <t>1.001,88</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>13/04/2026 07:00 a.m.</t>
+          <t>13/04/2026 09:00 a.m.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>29,25</t>
+          <t>31,69</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -744,24 +744,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,32</t>
+          <t>0,78</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.000,76</t>
+          <t>1.001,82</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>13/04/2026 06:00 a.m.</t>
+          <t>13/04/2026 08:00 a.m.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>28,51</t>
+          <t>30,87</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -771,24 +771,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>999,89</t>
+          <t>1.001,49</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>13/04/2026 05:00 a.m.</t>
+          <t>13/04/2026 07:00 a.m.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28,49</t>
+          <t>29,25</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -798,24 +798,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>999,42</t>
+          <t>1.000,76</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>13/04/2026 04:00 a.m.</t>
+          <t>13/04/2026 06:00 a.m.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>28,28</t>
+          <t>28,51</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -825,24 +825,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0,00</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>999,10</t>
+          <t>999,89</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>13/04/2026 03:00 a.m.</t>
+          <t>13/04/2026 05:00 a.m.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>28,06</t>
+          <t>28,49</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -857,19 +857,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>999,21</t>
+          <t>999,42</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>13/04/2026 02:00 a.m.</t>
+          <t>13/04/2026 04:00 a.m.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>28,59</t>
+          <t>28,28</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -884,19 +884,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>999,73</t>
+          <t>999,10</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>13/04/2026 01:00 a.m.</t>
+          <t>13/04/2026 03:00 a.m.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>28,71</t>
+          <t>28,06</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -911,19 +911,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.000,26</t>
+          <t>999,21</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>13/04/2026 12:00 a.m.</t>
+          <t>13/04/2026 02:00 a.m.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>28,64</t>
+          <t>28,59</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -938,19 +938,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.000,94</t>
+          <t>999,73</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/04/2026 11:00 p.m.</t>
+          <t>13/04/2026 01:00 a.m.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>28,70</t>
+          <t>28,71</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -965,19 +965,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.001,40</t>
+          <t>1.000,26</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12/04/2026 10:00 p.m.</t>
+          <t>13/04/2026 12:00 a.m.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>28,91</t>
+          <t>28,64</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -992,19 +992,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.001,65</t>
+          <t>1.000,94</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12/04/2026 09:00 p.m.</t>
+          <t>12/04/2026 11:00 p.m.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>29,29</t>
+          <t>28,70</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1019,19 +1019,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.001,33</t>
+          <t>1.001,40</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/04/2026 08:00 p.m.</t>
+          <t>12/04/2026 10:00 p.m.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>29,73</t>
+          <t>28,91</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1046,19 +1046,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.001,15</t>
+          <t>1.001,65</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/04/2026 07:00 p.m.</t>
+          <t>12/04/2026 09:00 p.m.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>30,35</t>
+          <t>29,29</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1073,19 +1073,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.000,43</t>
+          <t>1.001,33</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/04/2026 06:00 p.m.</t>
+          <t>12/04/2026 08:00 p.m.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>31,93</t>
+          <t>29,73</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1095,24 +1095,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0,16</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>999,54</t>
+          <t>1.001,15</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12/04/2026 05:00 p.m.</t>
+          <t>12/04/2026 07:00 p.m.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>33,52</t>
+          <t>30,35</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0,41</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>998,68</t>
+          <t>1.000,43</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13/04/2026 05:42:27 p.m.</t>
+          <t>13/04/2026 07:52:27 p.m.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>